<commit_message>
add supplementary table 1A script, table 1b, and zip files
</commit_message>
<xml_diff>
--- a/library_survey_supplementary_materials/supp_table_1b_GRCh38_vs_T2T_21_unmapped_genes.xlsx
+++ b/library_survey_supplementary_materials/supp_table_1b_GRCh38_vs_T2T_21_unmapped_genes.xlsx
@@ -1,175 +1,179 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\CRISPR-KO-library-survey\library_survey_supplementary_materials\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B1DD45-4179-44F1-8A0B-5B511DD3CA25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
-  <si>
-    <t xml:space="preserve">gene_id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grch38_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grch38_chromosome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">t2t_chm13_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">t2t_chromosome</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reason_for_loss</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CD200R1L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reclassified as pseudogene in T2T-CHM13v2.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">protein-coding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transcribed_pseudogene</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-annotated as transcribed_pseudogene in T2T-CHM13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No curated RefSeq (NP_) transcript in T2T-CHM13v2.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">protein-coding gene model (Gnomon XP_ only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gnomon-predicted (XP_) only, no curated NP_ transcript (symbol also resolves to a separate non-coding/partial GFF record: gene-CLN3, biotype other)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CYP4B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EFCAB13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GSTM2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gnomon-predicted (XP_) only, no curated NP_ transcript</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KCTD16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRT24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRT81</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRTAP5-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not annotated in T2T-CHM13v2.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Absent - no gene model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Locus not annotated in T2T-CHM13v2.0 RefSeq (GCF_009914755.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRTAP5-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRTAP9-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEO1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MS4A14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLA2G10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRSS48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIGLEC5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPRR3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAS2R43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBCD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UPK3BL1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZNF681</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="49">
+  <si>
+    <t>gene_id</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>grch38_status</t>
+  </si>
+  <si>
+    <t>grch38_chromosome</t>
+  </si>
+  <si>
+    <t>t2t_chm13_status</t>
+  </si>
+  <si>
+    <t>t2t_chromosome</t>
+  </si>
+  <si>
+    <t>reason_for_loss</t>
+  </si>
+  <si>
+    <t>CD200R1L</t>
+  </si>
+  <si>
+    <t>Reclassified as pseudogene in T2T-CHM13v2.0</t>
+  </si>
+  <si>
+    <t>protein-coding</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>transcribed_pseudogene</t>
+  </si>
+  <si>
+    <t>Re-annotated as transcribed_pseudogene in T2T-CHM13</t>
+  </si>
+  <si>
+    <t>CLN3</t>
+  </si>
+  <si>
+    <t>No curated RefSeq (NP_) transcript in T2T-CHM13v2.0</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>protein-coding gene model (Gnomon XP_ only)</t>
+  </si>
+  <si>
+    <t>CYP4B1</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>EFCAB13</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>GSTM2</t>
+  </si>
+  <si>
+    <t>Gnomon-predicted (XP_) only, no curated NP_ transcript</t>
+  </si>
+  <si>
+    <t>KCTD16</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>KRT24</t>
+  </si>
+  <si>
+    <t>KRT81</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>KRTAP5-1</t>
+  </si>
+  <si>
+    <t>Not annotated in T2T-CHM13v2.0</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>Absent - no gene model</t>
+  </si>
+  <si>
+    <t>Locus not annotated in T2T-CHM13v2.0 RefSeq (GCF_009914755.1)</t>
+  </si>
+  <si>
+    <t>KRTAP5-10</t>
+  </si>
+  <si>
+    <t>KRTAP9-7</t>
+  </si>
+  <si>
+    <t>LEO1</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>MS4A14</t>
+  </si>
+  <si>
+    <t>PLA2G10</t>
+  </si>
+  <si>
+    <t>PRSS48</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>SIGLEC5</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>SPRR3</t>
+  </si>
+  <si>
+    <t>TAS2R43</t>
+  </si>
+  <si>
+    <t>TBCD</t>
+  </si>
+  <si>
+    <t>UPK3BL1</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>ZNF681</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -205,6 +209,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -486,11 +499,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,7 +526,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -536,7 +549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -556,12 +569,12 @@
         <v>15</v>
       </c>
       <c r="G3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -570,21 +583,21 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
@@ -593,21 +606,21 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -616,21 +629,21 @@
         <v>9</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
         <v>16</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>24</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
@@ -639,21 +652,21 @@
         <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
         <v>16</v>
       </c>
       <c r="F7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>25</v>
-      </c>
-      <c r="G7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>26</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
@@ -662,21 +675,21 @@
         <v>9</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -685,63 +698,61 @@
         <v>9</v>
       </c>
       <c r="D9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>31</v>
       </c>
-      <c r="E10" t="s">
+      <c r="G10" t="s">
         <v>32</v>
       </c>
-      <c r="F10"/>
-      <c r="G10" t="s">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>34</v>
-      </c>
-      <c r="B11" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" t="s">
-        <v>32</v>
-      </c>
-      <c r="F11"/>
-      <c r="G11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>35</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -750,21 +761,21 @@
         <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E12" t="s">
         <v>16</v>
       </c>
       <c r="F12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
         <v>8</v>
@@ -773,21 +784,21 @@
         <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E13" t="s">
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B14" t="s">
         <v>8</v>
@@ -796,24 +807,24 @@
         <v>9</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
@@ -822,16 +833,15 @@
         <v>15</v>
       </c>
       <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" t="s">
         <v>32</v>
       </c>
-      <c r="F15"/>
-      <c r="G15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B16" t="s">
         <v>8</v>
@@ -840,21 +850,21 @@
         <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E16" t="s">
         <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
@@ -863,21 +873,21 @@
         <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
         <v>16</v>
       </c>
       <c r="F17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>43</v>
-      </c>
-      <c r="G17" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>44</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
@@ -886,42 +896,41 @@
         <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
         <v>16</v>
       </c>
       <c r="F18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G18" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>45</v>
-      </c>
-      <c r="B19" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D19" t="s">
-        <v>28</v>
-      </c>
-      <c r="E19" t="s">
-        <v>32</v>
-      </c>
-      <c r="F19"/>
-      <c r="G19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>46</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
@@ -930,42 +939,41 @@
         <v>9</v>
       </c>
       <c r="D20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E20" t="s">
         <v>16</v>
       </c>
       <c r="F20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" t="s">
         <v>47</v>
       </c>
-      <c r="B21" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
+        <v>31</v>
+      </c>
+      <c r="G21" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>48</v>
-      </c>
-      <c r="E21" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21"/>
-      <c r="G21" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>49</v>
       </c>
       <c r="B22" t="s">
         <v>8</v>
@@ -974,13 +982,13 @@
         <v>9</v>
       </c>
       <c r="D22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E22" t="s">
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G22" t="s">
         <v>12</v>
@@ -988,6 +996,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>